<commit_message>
Product Name is fetched according to Product ID from Sheet2  using xlookup formula
</commit_message>
<xml_diff>
--- a/Day 3/Day3_Practice_Data.xlsx
+++ b/Day 3/Day3_Practice_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD32042D-83C3-4E02-B382-BECD9AF73AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90E8D214-FAEA-409C-8449-B0EF2286A107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{2C26B9A5-BE97-4C69-AF28-CEF3FE580AAE}"/>
   </bookViews>
@@ -691,7 +691,9 @@
   <dimension ref="A1:J41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="9" width="13.77734375" customWidth="1"/>
+    <col min="1" max="5" width="13.77734375" customWidth="1"/>
+    <col min="6" max="6" width="17.5546875" customWidth="1"/>
+    <col min="7" max="9" width="13.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -739,7 +741,10 @@
       <c r="E2" s="5">
         <v>4</v>
       </c>
-      <c r="F2" s="5"/>
+      <c r="F2" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C2,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Laptop Pro</v>
+      </c>
       <c r="G2" s="5"/>
       <c r="H2" s="9"/>
       <c r="I2" s="5"/>
@@ -761,7 +766,10 @@
       <c r="E3" s="5">
         <v>1</v>
       </c>
-      <c r="F3" s="5"/>
+      <c r="F3" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C3,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Wireless Mouse</v>
+      </c>
       <c r="G3" s="5"/>
       <c r="H3" s="9"/>
       <c r="I3" s="5"/>
@@ -783,7 +791,10 @@
       <c r="E4" s="5">
         <v>9</v>
       </c>
-      <c r="F4" s="5"/>
+      <c r="F4" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C4,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Office Chair</v>
+      </c>
       <c r="G4" s="5"/>
       <c r="H4" s="9"/>
       <c r="I4" s="5"/>
@@ -805,7 +816,10 @@
       <c r="E5" s="5">
         <v>8</v>
       </c>
-      <c r="F5" s="5"/>
+      <c r="F5" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C5,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Notebook Set</v>
+      </c>
       <c r="G5" s="5"/>
       <c r="H5" s="9"/>
       <c r="I5" s="5"/>
@@ -827,7 +841,10 @@
       <c r="E6" s="5">
         <v>8</v>
       </c>
-      <c r="F6" s="5"/>
+      <c r="F6" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C6,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>USB-C Hub</v>
+      </c>
       <c r="G6" s="5"/>
       <c r="H6" s="9"/>
       <c r="I6" s="5"/>
@@ -849,7 +866,10 @@
       <c r="E7" s="5">
         <v>5</v>
       </c>
-      <c r="F7" s="5"/>
+      <c r="F7" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C7,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Standing Desk</v>
+      </c>
       <c r="G7" s="5"/>
       <c r="H7" s="9"/>
       <c r="I7" s="5"/>
@@ -871,7 +891,10 @@
       <c r="E8" s="5">
         <v>5</v>
       </c>
-      <c r="F8" s="5"/>
+      <c r="F8" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C8,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Standing Desk</v>
+      </c>
       <c r="G8" s="5"/>
       <c r="H8" s="9"/>
       <c r="I8" s="5"/>
@@ -893,7 +916,10 @@
       <c r="E9" s="5">
         <v>4</v>
       </c>
-      <c r="F9" s="5"/>
+      <c r="F9" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C9,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Webcam HD</v>
+      </c>
       <c r="G9" s="5"/>
       <c r="H9" s="9"/>
       <c r="I9" s="5"/>
@@ -915,7 +941,10 @@
       <c r="E10" s="5">
         <v>3</v>
       </c>
-      <c r="F10" s="5"/>
+      <c r="F10" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C10,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Monitor 27"</v>
+      </c>
       <c r="G10" s="5"/>
       <c r="H10" s="9"/>
       <c r="I10" s="5"/>
@@ -937,7 +966,10 @@
       <c r="E11" s="5">
         <v>19</v>
       </c>
-      <c r="F11" s="5"/>
+      <c r="F11" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C11,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Desk Lamp LED</v>
+      </c>
       <c r="G11" s="5"/>
       <c r="H11" s="9"/>
       <c r="I11" s="5"/>
@@ -959,7 +991,10 @@
       <c r="E12" s="5">
         <v>14</v>
       </c>
-      <c r="F12" s="5"/>
+      <c r="F12" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C12,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Laptop Pro</v>
+      </c>
       <c r="G12" s="5"/>
       <c r="H12" s="9"/>
       <c r="I12" s="5"/>
@@ -981,7 +1016,10 @@
       <c r="E13" s="5">
         <v>2</v>
       </c>
-      <c r="F13" s="5"/>
+      <c r="F13" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C13,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Wireless Mouse</v>
+      </c>
       <c r="G13" s="5"/>
       <c r="H13" s="9"/>
       <c r="I13" s="5"/>
@@ -1003,7 +1041,10 @@
       <c r="E14" s="5">
         <v>1</v>
       </c>
-      <c r="F14" s="5"/>
+      <c r="F14" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C14,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Office Chair</v>
+      </c>
       <c r="G14" s="5"/>
       <c r="H14" s="9"/>
       <c r="I14" s="5"/>
@@ -1025,7 +1066,10 @@
       <c r="E15" s="5">
         <v>3</v>
       </c>
-      <c r="F15" s="5"/>
+      <c r="F15" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C15,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Notebook Set</v>
+      </c>
       <c r="G15" s="5"/>
       <c r="H15" s="9"/>
       <c r="I15" s="5"/>
@@ -1047,7 +1091,10 @@
       <c r="E16" s="5">
         <v>7</v>
       </c>
-      <c r="F16" s="5"/>
+      <c r="F16" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C16,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>USB-C Hub</v>
+      </c>
       <c r="G16" s="5"/>
       <c r="H16" s="9"/>
       <c r="I16" s="5"/>
@@ -1069,7 +1116,10 @@
       <c r="E17" s="5">
         <v>17</v>
       </c>
-      <c r="F17" s="5"/>
+      <c r="F17" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C17,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Webcam HD</v>
+      </c>
       <c r="G17" s="5"/>
       <c r="H17" s="9"/>
       <c r="I17" s="5"/>
@@ -1091,7 +1141,10 @@
       <c r="E18" s="5">
         <v>20</v>
       </c>
-      <c r="F18" s="5"/>
+      <c r="F18" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C18,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Pen Drive 128GB</v>
+      </c>
       <c r="G18" s="5"/>
       <c r="H18" s="9"/>
       <c r="I18" s="5"/>
@@ -1113,7 +1166,10 @@
       <c r="E19" s="5">
         <v>1</v>
       </c>
-      <c r="F19" s="5"/>
+      <c r="F19" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C19,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Monitor 27"</v>
+      </c>
       <c r="G19" s="5"/>
       <c r="H19" s="9"/>
       <c r="I19" s="5"/>
@@ -1135,7 +1191,10 @@
       <c r="E20" s="5">
         <v>18</v>
       </c>
-      <c r="F20" s="5"/>
+      <c r="F20" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C20,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Desk Lamp LED</v>
+      </c>
       <c r="G20" s="5"/>
       <c r="H20" s="9"/>
       <c r="I20" s="5"/>
@@ -1157,7 +1216,10 @@
       <c r="E21" s="5">
         <v>7</v>
       </c>
-      <c r="F21" s="5"/>
+      <c r="F21" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C21,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Laptop Pro</v>
+      </c>
       <c r="G21" s="5"/>
       <c r="H21" s="9"/>
       <c r="I21" s="5"/>
@@ -1179,7 +1241,10 @@
       <c r="E22" s="5">
         <v>7</v>
       </c>
-      <c r="F22" s="5"/>
+      <c r="F22" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C22,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Laptop Pro</v>
+      </c>
       <c r="G22" s="5"/>
       <c r="H22" s="9"/>
       <c r="I22" s="5"/>
@@ -1201,7 +1266,10 @@
       <c r="E23" s="5">
         <v>18</v>
       </c>
-      <c r="F23" s="5"/>
+      <c r="F23" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C23,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Wireless Mouse</v>
+      </c>
       <c r="G23" s="5"/>
       <c r="H23" s="9"/>
       <c r="I23" s="5"/>
@@ -1223,7 +1291,10 @@
       <c r="E24" s="5">
         <v>14</v>
       </c>
-      <c r="F24" s="5"/>
+      <c r="F24" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C24,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Office Chair</v>
+      </c>
       <c r="G24" s="5"/>
       <c r="H24" s="9"/>
       <c r="I24" s="5"/>
@@ -1245,7 +1316,10 @@
       <c r="E25" s="5">
         <v>15</v>
       </c>
-      <c r="F25" s="5"/>
+      <c r="F25" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C25,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>USB-C Hub</v>
+      </c>
       <c r="G25" s="5"/>
       <c r="H25" s="9"/>
       <c r="I25" s="5"/>
@@ -1267,7 +1341,10 @@
       <c r="E26" s="5">
         <v>19</v>
       </c>
-      <c r="F26" s="5"/>
+      <c r="F26" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C26,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Standing Desk</v>
+      </c>
       <c r="G26" s="5"/>
       <c r="H26" s="9"/>
       <c r="I26" s="5"/>
@@ -1289,7 +1366,10 @@
       <c r="E27" s="5">
         <v>9</v>
       </c>
-      <c r="F27" s="5"/>
+      <c r="F27" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C27,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Webcam HD</v>
+      </c>
       <c r="G27" s="5"/>
       <c r="H27" s="9"/>
       <c r="I27" s="5"/>
@@ -1311,7 +1391,10 @@
       <c r="E28" s="5">
         <v>1</v>
       </c>
-      <c r="F28" s="5"/>
+      <c r="F28" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C28,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Pen Drive 128GB</v>
+      </c>
       <c r="G28" s="5"/>
       <c r="H28" s="9"/>
       <c r="I28" s="5"/>
@@ -1333,7 +1416,10 @@
       <c r="E29" s="5">
         <v>6</v>
       </c>
-      <c r="F29" s="5"/>
+      <c r="F29" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C29,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Monitor 27"</v>
+      </c>
       <c r="G29" s="5"/>
       <c r="H29" s="9"/>
       <c r="I29" s="5"/>
@@ -1355,7 +1441,10 @@
       <c r="E30" s="5">
         <v>14</v>
       </c>
-      <c r="F30" s="5"/>
+      <c r="F30" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C30,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Desk Lamp LED</v>
+      </c>
       <c r="G30" s="5"/>
       <c r="H30" s="9"/>
       <c r="I30" s="5"/>
@@ -1377,7 +1466,10 @@
       <c r="E31" s="5">
         <v>11</v>
       </c>
-      <c r="F31" s="5"/>
+      <c r="F31" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C31,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Laptop Pro</v>
+      </c>
       <c r="G31" s="5"/>
       <c r="H31" s="9"/>
       <c r="I31" s="5"/>
@@ -1399,7 +1491,10 @@
       <c r="E32" s="5">
         <v>9</v>
       </c>
-      <c r="F32" s="5"/>
+      <c r="F32" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C32,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Wireless Mouse</v>
+      </c>
       <c r="G32" s="5"/>
       <c r="H32" s="9"/>
       <c r="I32" s="5"/>
@@ -1421,7 +1516,10 @@
       <c r="E33" s="5">
         <v>5</v>
       </c>
-      <c r="F33" s="5"/>
+      <c r="F33" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C33,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Office Chair</v>
+      </c>
       <c r="G33" s="5"/>
       <c r="H33" s="9"/>
       <c r="I33" s="5"/>
@@ -1443,7 +1541,10 @@
       <c r="E34" s="5">
         <v>11</v>
       </c>
-      <c r="F34" s="5"/>
+      <c r="F34" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C34,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>USB-C Hub</v>
+      </c>
       <c r="G34" s="5"/>
       <c r="H34" s="9"/>
       <c r="I34" s="5"/>
@@ -1465,7 +1566,10 @@
       <c r="E35" s="5">
         <v>4</v>
       </c>
-      <c r="F35" s="5"/>
+      <c r="F35" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C35,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Standing Desk</v>
+      </c>
       <c r="G35" s="5"/>
       <c r="H35" s="9"/>
       <c r="I35" s="5"/>
@@ -1487,7 +1591,10 @@
       <c r="E36" s="5">
         <v>4</v>
       </c>
-      <c r="F36" s="5"/>
+      <c r="F36" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C36,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Standing Desk</v>
+      </c>
       <c r="G36" s="5"/>
       <c r="H36" s="9"/>
       <c r="I36" s="5"/>
@@ -1509,7 +1616,10 @@
       <c r="E37" s="5">
         <v>3</v>
       </c>
-      <c r="F37" s="5"/>
+      <c r="F37" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C37,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Webcam HD</v>
+      </c>
       <c r="G37" s="5"/>
       <c r="H37" s="9"/>
       <c r="I37" s="5"/>
@@ -1531,7 +1641,10 @@
       <c r="E38" s="5">
         <v>13</v>
       </c>
-      <c r="F38" s="5"/>
+      <c r="F38" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C38,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Pen Drive 128GB</v>
+      </c>
       <c r="G38" s="5"/>
       <c r="H38" s="9"/>
       <c r="I38" s="5"/>
@@ -1553,7 +1666,10 @@
       <c r="E39" s="5">
         <v>4</v>
       </c>
-      <c r="F39" s="5"/>
+      <c r="F39" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C39,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Monitor 27"</v>
+      </c>
       <c r="G39" s="5"/>
       <c r="H39" s="9"/>
       <c r="I39" s="5"/>
@@ -1575,7 +1691,10 @@
       <c r="E40" s="5">
         <v>12</v>
       </c>
-      <c r="F40" s="5"/>
+      <c r="F40" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C40,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Desk Lamp LED</v>
+      </c>
       <c r="G40" s="5"/>
       <c r="H40" s="9"/>
       <c r="I40" s="5"/>
@@ -1597,7 +1716,10 @@
       <c r="E41" s="5">
         <v>12</v>
       </c>
-      <c r="F41" s="5"/>
+      <c r="F41" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C41,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
+        <v>Laptop Pro</v>
+      </c>
       <c r="G41" s="5"/>
       <c r="H41" s="9"/>
       <c r="I41" s="5"/>

</xml_diff>

<commit_message>
Product Category is fetched according to Product ID from Sheet2  using xlookup formula
</commit_message>
<xml_diff>
--- a/Day 3/Day3_Practice_Data.xlsx
+++ b/Day 3/Day3_Practice_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90E8D214-FAEA-409C-8449-B0EF2286A107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45248EB8-5890-4E3D-9D34-38A98E47F815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{2C26B9A5-BE97-4C69-AF28-CEF3FE580AAE}"/>
   </bookViews>
@@ -745,7 +745,10 @@
         <f>_xlfn.XLOOKUP(C2,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Laptop Pro</v>
       </c>
-      <c r="G2" s="5"/>
+      <c r="G2" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C2,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H2" s="9"/>
       <c r="I2" s="5"/>
       <c r="J2" s="1"/>
@@ -770,7 +773,10 @@
         <f>_xlfn.XLOOKUP(C3,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Wireless Mouse</v>
       </c>
-      <c r="G3" s="5"/>
+      <c r="G3" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C3,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Accessories</v>
+      </c>
       <c r="H3" s="9"/>
       <c r="I3" s="5"/>
       <c r="J3" s="1"/>
@@ -795,7 +801,10 @@
         <f>_xlfn.XLOOKUP(C4,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Office Chair</v>
       </c>
-      <c r="G4" s="5"/>
+      <c r="G4" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C4,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H4" s="9"/>
       <c r="I4" s="5"/>
       <c r="J4" s="1"/>
@@ -820,7 +829,10 @@
         <f>_xlfn.XLOOKUP(C5,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Notebook Set</v>
       </c>
-      <c r="G5" s="5"/>
+      <c r="G5" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C5,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Stationery</v>
+      </c>
       <c r="H5" s="9"/>
       <c r="I5" s="5"/>
       <c r="J5" s="1"/>
@@ -845,7 +857,10 @@
         <f>_xlfn.XLOOKUP(C6,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>USB-C Hub</v>
       </c>
-      <c r="G6" s="5"/>
+      <c r="G6" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C6,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Accessories</v>
+      </c>
       <c r="H6" s="9"/>
       <c r="I6" s="5"/>
       <c r="J6" s="1"/>
@@ -870,7 +885,10 @@
         <f>_xlfn.XLOOKUP(C7,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Standing Desk</v>
       </c>
-      <c r="G7" s="5"/>
+      <c r="G7" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C7,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H7" s="9"/>
       <c r="I7" s="5"/>
       <c r="J7" s="1"/>
@@ -895,7 +913,10 @@
         <f>_xlfn.XLOOKUP(C8,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Standing Desk</v>
       </c>
-      <c r="G8" s="5"/>
+      <c r="G8" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C8,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H8" s="9"/>
       <c r="I8" s="5"/>
       <c r="J8" s="1"/>
@@ -920,7 +941,10 @@
         <f>_xlfn.XLOOKUP(C9,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Webcam HD</v>
       </c>
-      <c r="G9" s="5"/>
+      <c r="G9" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C9,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H9" s="9"/>
       <c r="I9" s="5"/>
       <c r="J9" s="1"/>
@@ -945,7 +969,10 @@
         <f>_xlfn.XLOOKUP(C10,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Monitor 27"</v>
       </c>
-      <c r="G10" s="5"/>
+      <c r="G10" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C10,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H10" s="9"/>
       <c r="I10" s="5"/>
       <c r="J10" s="1"/>
@@ -970,7 +997,10 @@
         <f>_xlfn.XLOOKUP(C11,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Desk Lamp LED</v>
       </c>
-      <c r="G11" s="5"/>
+      <c r="G11" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C11,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H11" s="9"/>
       <c r="I11" s="5"/>
       <c r="J11" s="1"/>
@@ -995,7 +1025,10 @@
         <f>_xlfn.XLOOKUP(C12,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Laptop Pro</v>
       </c>
-      <c r="G12" s="5"/>
+      <c r="G12" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C12,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H12" s="9"/>
       <c r="I12" s="5"/>
       <c r="J12" s="1"/>
@@ -1020,7 +1053,10 @@
         <f>_xlfn.XLOOKUP(C13,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Wireless Mouse</v>
       </c>
-      <c r="G13" s="5"/>
+      <c r="G13" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C13,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Accessories</v>
+      </c>
       <c r="H13" s="9"/>
       <c r="I13" s="5"/>
       <c r="J13" s="1"/>
@@ -1045,7 +1081,10 @@
         <f>_xlfn.XLOOKUP(C14,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Office Chair</v>
       </c>
-      <c r="G14" s="5"/>
+      <c r="G14" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C14,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H14" s="9"/>
       <c r="I14" s="5"/>
       <c r="J14" s="1"/>
@@ -1070,7 +1109,10 @@
         <f>_xlfn.XLOOKUP(C15,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Notebook Set</v>
       </c>
-      <c r="G15" s="5"/>
+      <c r="G15" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C15,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Stationery</v>
+      </c>
       <c r="H15" s="9"/>
       <c r="I15" s="5"/>
       <c r="J15" s="1"/>
@@ -1095,7 +1137,10 @@
         <f>_xlfn.XLOOKUP(C16,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>USB-C Hub</v>
       </c>
-      <c r="G16" s="5"/>
+      <c r="G16" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C16,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Accessories</v>
+      </c>
       <c r="H16" s="9"/>
       <c r="I16" s="5"/>
       <c r="J16" s="1"/>
@@ -1120,7 +1165,10 @@
         <f>_xlfn.XLOOKUP(C17,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Webcam HD</v>
       </c>
-      <c r="G17" s="5"/>
+      <c r="G17" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C17,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H17" s="9"/>
       <c r="I17" s="5"/>
       <c r="J17" s="1"/>
@@ -1145,7 +1193,10 @@
         <f>_xlfn.XLOOKUP(C18,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Pen Drive 128GB</v>
       </c>
-      <c r="G18" s="5"/>
+      <c r="G18" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C18,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Accessories</v>
+      </c>
       <c r="H18" s="9"/>
       <c r="I18" s="5"/>
       <c r="J18" s="1"/>
@@ -1170,7 +1221,10 @@
         <f>_xlfn.XLOOKUP(C19,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Monitor 27"</v>
       </c>
-      <c r="G19" s="5"/>
+      <c r="G19" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C19,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H19" s="9"/>
       <c r="I19" s="5"/>
       <c r="J19" s="1"/>
@@ -1195,7 +1249,10 @@
         <f>_xlfn.XLOOKUP(C20,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Desk Lamp LED</v>
       </c>
-      <c r="G20" s="5"/>
+      <c r="G20" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C20,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H20" s="9"/>
       <c r="I20" s="5"/>
       <c r="J20" s="1"/>
@@ -1220,7 +1277,10 @@
         <f>_xlfn.XLOOKUP(C21,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Laptop Pro</v>
       </c>
-      <c r="G21" s="5"/>
+      <c r="G21" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C21,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H21" s="9"/>
       <c r="I21" s="5"/>
       <c r="J21" s="1"/>
@@ -1245,7 +1305,10 @@
         <f>_xlfn.XLOOKUP(C22,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Laptop Pro</v>
       </c>
-      <c r="G22" s="5"/>
+      <c r="G22" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C22,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H22" s="9"/>
       <c r="I22" s="5"/>
       <c r="J22" s="1"/>
@@ -1270,7 +1333,10 @@
         <f>_xlfn.XLOOKUP(C23,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Wireless Mouse</v>
       </c>
-      <c r="G23" s="5"/>
+      <c r="G23" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C23,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Accessories</v>
+      </c>
       <c r="H23" s="9"/>
       <c r="I23" s="5"/>
       <c r="J23" s="1"/>
@@ -1295,7 +1361,10 @@
         <f>_xlfn.XLOOKUP(C24,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Office Chair</v>
       </c>
-      <c r="G24" s="5"/>
+      <c r="G24" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C24,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H24" s="9"/>
       <c r="I24" s="5"/>
       <c r="J24" s="1"/>
@@ -1320,7 +1389,10 @@
         <f>_xlfn.XLOOKUP(C25,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>USB-C Hub</v>
       </c>
-      <c r="G25" s="5"/>
+      <c r="G25" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C25,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Accessories</v>
+      </c>
       <c r="H25" s="9"/>
       <c r="I25" s="5"/>
       <c r="J25" s="1"/>
@@ -1345,7 +1417,10 @@
         <f>_xlfn.XLOOKUP(C26,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Standing Desk</v>
       </c>
-      <c r="G26" s="5"/>
+      <c r="G26" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C26,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H26" s="9"/>
       <c r="I26" s="5"/>
       <c r="J26" s="1"/>
@@ -1370,7 +1445,10 @@
         <f>_xlfn.XLOOKUP(C27,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Webcam HD</v>
       </c>
-      <c r="G27" s="5"/>
+      <c r="G27" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C27,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H27" s="9"/>
       <c r="I27" s="5"/>
       <c r="J27" s="1"/>
@@ -1395,7 +1473,10 @@
         <f>_xlfn.XLOOKUP(C28,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Pen Drive 128GB</v>
       </c>
-      <c r="G28" s="5"/>
+      <c r="G28" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C28,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Accessories</v>
+      </c>
       <c r="H28" s="9"/>
       <c r="I28" s="5"/>
       <c r="J28" s="1"/>
@@ -1420,7 +1501,10 @@
         <f>_xlfn.XLOOKUP(C29,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Monitor 27"</v>
       </c>
-      <c r="G29" s="5"/>
+      <c r="G29" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C29,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H29" s="9"/>
       <c r="I29" s="5"/>
       <c r="J29" s="1"/>
@@ -1445,7 +1529,10 @@
         <f>_xlfn.XLOOKUP(C30,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Desk Lamp LED</v>
       </c>
-      <c r="G30" s="5"/>
+      <c r="G30" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C30,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H30" s="9"/>
       <c r="I30" s="5"/>
       <c r="J30" s="1"/>
@@ -1470,7 +1557,10 @@
         <f>_xlfn.XLOOKUP(C31,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Laptop Pro</v>
       </c>
-      <c r="G31" s="5"/>
+      <c r="G31" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C31,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H31" s="9"/>
       <c r="I31" s="5"/>
       <c r="J31" s="1"/>
@@ -1495,7 +1585,10 @@
         <f>_xlfn.XLOOKUP(C32,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Wireless Mouse</v>
       </c>
-      <c r="G32" s="5"/>
+      <c r="G32" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C32,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Accessories</v>
+      </c>
       <c r="H32" s="9"/>
       <c r="I32" s="5"/>
       <c r="J32" s="1"/>
@@ -1520,7 +1613,10 @@
         <f>_xlfn.XLOOKUP(C33,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Office Chair</v>
       </c>
-      <c r="G33" s="5"/>
+      <c r="G33" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C33,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H33" s="9"/>
       <c r="I33" s="5"/>
       <c r="J33" s="1"/>
@@ -1545,7 +1641,10 @@
         <f>_xlfn.XLOOKUP(C34,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>USB-C Hub</v>
       </c>
-      <c r="G34" s="5"/>
+      <c r="G34" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C34,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Accessories</v>
+      </c>
       <c r="H34" s="9"/>
       <c r="I34" s="5"/>
       <c r="J34" s="1"/>
@@ -1570,7 +1669,10 @@
         <f>_xlfn.XLOOKUP(C35,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Standing Desk</v>
       </c>
-      <c r="G35" s="5"/>
+      <c r="G35" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C35,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H35" s="9"/>
       <c r="I35" s="5"/>
       <c r="J35" s="1"/>
@@ -1595,7 +1697,10 @@
         <f>_xlfn.XLOOKUP(C36,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Standing Desk</v>
       </c>
-      <c r="G36" s="5"/>
+      <c r="G36" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C36,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H36" s="9"/>
       <c r="I36" s="5"/>
       <c r="J36" s="1"/>
@@ -1620,7 +1725,10 @@
         <f>_xlfn.XLOOKUP(C37,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Webcam HD</v>
       </c>
-      <c r="G37" s="5"/>
+      <c r="G37" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C37,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H37" s="9"/>
       <c r="I37" s="5"/>
       <c r="J37" s="1"/>
@@ -1645,7 +1753,10 @@
         <f>_xlfn.XLOOKUP(C38,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Pen Drive 128GB</v>
       </c>
-      <c r="G38" s="5"/>
+      <c r="G38" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C38,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Accessories</v>
+      </c>
       <c r="H38" s="9"/>
       <c r="I38" s="5"/>
       <c r="J38" s="1"/>
@@ -1670,7 +1781,10 @@
         <f>_xlfn.XLOOKUP(C39,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Monitor 27"</v>
       </c>
-      <c r="G39" s="5"/>
+      <c r="G39" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C39,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H39" s="9"/>
       <c r="I39" s="5"/>
       <c r="J39" s="1"/>
@@ -1695,7 +1809,10 @@
         <f>_xlfn.XLOOKUP(C40,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Desk Lamp LED</v>
       </c>
-      <c r="G40" s="5"/>
+      <c r="G40" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C40,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Furniture</v>
+      </c>
       <c r="H40" s="9"/>
       <c r="I40" s="5"/>
       <c r="J40" s="1"/>
@@ -1720,7 +1837,10 @@
         <f>_xlfn.XLOOKUP(C41,Sheet2!$A$2:$A$11,Sheet2!$B$2:$B$11)</f>
         <v>Laptop Pro</v>
       </c>
-      <c r="G41" s="5"/>
+      <c r="G41" s="5" t="str">
+        <f>_xlfn.XLOOKUP(C41,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
+        <v>Electronics</v>
+      </c>
       <c r="H41" s="9"/>
       <c r="I41" s="5"/>
       <c r="J41" s="1"/>

</xml_diff>

<commit_message>
Product Brand is fetched according to Product ID from Sheet2  using xlookup formula
</commit_message>
<xml_diff>
--- a/Day 3/Day3_Practice_Data.xlsx
+++ b/Day 3/Day3_Practice_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45248EB8-5890-4E3D-9D34-38A98E47F815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{019F2CB7-FC5B-45D7-B083-5541DA50C83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{2C26B9A5-BE97-4C69-AF28-CEF3FE580AAE}"/>
   </bookViews>
@@ -749,7 +749,10 @@
         <f>_xlfn.XLOOKUP(C2,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H2" s="9"/>
+      <c r="H2" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C2,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I2" s="5"/>
       <c r="J2" s="1"/>
     </row>
@@ -777,7 +780,10 @@
         <f>_xlfn.XLOOKUP(C3,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Accessories</v>
       </c>
-      <c r="H3" s="9"/>
+      <c r="H3" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C3,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I3" s="5"/>
       <c r="J3" s="1"/>
     </row>
@@ -805,7 +811,10 @@
         <f>_xlfn.XLOOKUP(C4,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H4" s="9"/>
+      <c r="H4" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C4,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I4" s="5"/>
       <c r="J4" s="1"/>
     </row>
@@ -833,7 +842,10 @@
         <f>_xlfn.XLOOKUP(C5,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Stationery</v>
       </c>
-      <c r="H5" s="9"/>
+      <c r="H5" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C5,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>WriteRight</v>
+      </c>
       <c r="I5" s="5"/>
       <c r="J5" s="1"/>
     </row>
@@ -861,7 +873,10 @@
         <f>_xlfn.XLOOKUP(C6,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Accessories</v>
       </c>
-      <c r="H6" s="9"/>
+      <c r="H6" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C6,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I6" s="5"/>
       <c r="J6" s="1"/>
     </row>
@@ -889,7 +904,10 @@
         <f>_xlfn.XLOOKUP(C7,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H7" s="9"/>
+      <c r="H7" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C7,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I7" s="5"/>
       <c r="J7" s="1"/>
     </row>
@@ -917,7 +935,10 @@
         <f>_xlfn.XLOOKUP(C8,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H8" s="9"/>
+      <c r="H8" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C8,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I8" s="5"/>
       <c r="J8" s="1"/>
     </row>
@@ -945,7 +966,10 @@
         <f>_xlfn.XLOOKUP(C9,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H9" s="9"/>
+      <c r="H9" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C9,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I9" s="5"/>
       <c r="J9" s="1"/>
     </row>
@@ -973,7 +997,10 @@
         <f>_xlfn.XLOOKUP(C10,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H10" s="9"/>
+      <c r="H10" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C10,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I10" s="5"/>
       <c r="J10" s="1"/>
     </row>
@@ -1001,7 +1028,10 @@
         <f>_xlfn.XLOOKUP(C11,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H11" s="9"/>
+      <c r="H11" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C11,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I11" s="5"/>
       <c r="J11" s="1"/>
     </row>
@@ -1029,7 +1059,10 @@
         <f>_xlfn.XLOOKUP(C12,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H12" s="9"/>
+      <c r="H12" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C12,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I12" s="5"/>
       <c r="J12" s="1"/>
     </row>
@@ -1057,7 +1090,10 @@
         <f>_xlfn.XLOOKUP(C13,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Accessories</v>
       </c>
-      <c r="H13" s="9"/>
+      <c r="H13" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C13,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I13" s="5"/>
       <c r="J13" s="1"/>
     </row>
@@ -1085,7 +1121,10 @@
         <f>_xlfn.XLOOKUP(C14,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H14" s="9"/>
+      <c r="H14" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C14,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I14" s="5"/>
       <c r="J14" s="1"/>
     </row>
@@ -1113,7 +1152,10 @@
         <f>_xlfn.XLOOKUP(C15,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Stationery</v>
       </c>
-      <c r="H15" s="9"/>
+      <c r="H15" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C15,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>WriteRight</v>
+      </c>
       <c r="I15" s="5"/>
       <c r="J15" s="1"/>
     </row>
@@ -1141,7 +1183,10 @@
         <f>_xlfn.XLOOKUP(C16,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Accessories</v>
       </c>
-      <c r="H16" s="9"/>
+      <c r="H16" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C16,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I16" s="5"/>
       <c r="J16" s="1"/>
     </row>
@@ -1169,7 +1214,10 @@
         <f>_xlfn.XLOOKUP(C17,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H17" s="9"/>
+      <c r="H17" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C17,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I17" s="5"/>
       <c r="J17" s="1"/>
     </row>
@@ -1197,7 +1245,10 @@
         <f>_xlfn.XLOOKUP(C18,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Accessories</v>
       </c>
-      <c r="H18" s="9"/>
+      <c r="H18" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C18,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>StorePro</v>
+      </c>
       <c r="I18" s="5"/>
       <c r="J18" s="1"/>
     </row>
@@ -1225,7 +1276,10 @@
         <f>_xlfn.XLOOKUP(C19,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H19" s="9"/>
+      <c r="H19" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C19,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I19" s="5"/>
       <c r="J19" s="1"/>
     </row>
@@ -1253,7 +1307,10 @@
         <f>_xlfn.XLOOKUP(C20,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H20" s="9"/>
+      <c r="H20" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C20,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I20" s="5"/>
       <c r="J20" s="1"/>
     </row>
@@ -1281,7 +1338,10 @@
         <f>_xlfn.XLOOKUP(C21,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H21" s="9"/>
+      <c r="H21" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C21,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I21" s="5"/>
       <c r="J21" s="1"/>
     </row>
@@ -1309,7 +1369,10 @@
         <f>_xlfn.XLOOKUP(C22,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H22" s="9"/>
+      <c r="H22" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C22,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I22" s="5"/>
       <c r="J22" s="1"/>
     </row>
@@ -1337,7 +1400,10 @@
         <f>_xlfn.XLOOKUP(C23,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Accessories</v>
       </c>
-      <c r="H23" s="9"/>
+      <c r="H23" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C23,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I23" s="5"/>
       <c r="J23" s="1"/>
     </row>
@@ -1365,7 +1431,10 @@
         <f>_xlfn.XLOOKUP(C24,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H24" s="9"/>
+      <c r="H24" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C24,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I24" s="5"/>
       <c r="J24" s="1"/>
     </row>
@@ -1393,7 +1462,10 @@
         <f>_xlfn.XLOOKUP(C25,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Accessories</v>
       </c>
-      <c r="H25" s="9"/>
+      <c r="H25" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C25,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I25" s="5"/>
       <c r="J25" s="1"/>
     </row>
@@ -1421,7 +1493,10 @@
         <f>_xlfn.XLOOKUP(C26,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H26" s="9"/>
+      <c r="H26" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C26,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I26" s="5"/>
       <c r="J26" s="1"/>
     </row>
@@ -1449,7 +1524,10 @@
         <f>_xlfn.XLOOKUP(C27,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H27" s="9"/>
+      <c r="H27" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C27,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I27" s="5"/>
       <c r="J27" s="1"/>
     </row>
@@ -1477,7 +1555,10 @@
         <f>_xlfn.XLOOKUP(C28,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Accessories</v>
       </c>
-      <c r="H28" s="9"/>
+      <c r="H28" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C28,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>StorePro</v>
+      </c>
       <c r="I28" s="5"/>
       <c r="J28" s="1"/>
     </row>
@@ -1505,7 +1586,10 @@
         <f>_xlfn.XLOOKUP(C29,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H29" s="9"/>
+      <c r="H29" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C29,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I29" s="5"/>
       <c r="J29" s="1"/>
     </row>
@@ -1533,7 +1617,10 @@
         <f>_xlfn.XLOOKUP(C30,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H30" s="9"/>
+      <c r="H30" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C30,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I30" s="5"/>
       <c r="J30" s="1"/>
     </row>
@@ -1561,7 +1648,10 @@
         <f>_xlfn.XLOOKUP(C31,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H31" s="9"/>
+      <c r="H31" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C31,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I31" s="5"/>
       <c r="J31" s="1"/>
     </row>
@@ -1589,7 +1679,10 @@
         <f>_xlfn.XLOOKUP(C32,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Accessories</v>
       </c>
-      <c r="H32" s="9"/>
+      <c r="H32" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C32,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I32" s="5"/>
       <c r="J32" s="1"/>
     </row>
@@ -1617,7 +1710,10 @@
         <f>_xlfn.XLOOKUP(C33,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H33" s="9"/>
+      <c r="H33" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C33,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I33" s="5"/>
       <c r="J33" s="1"/>
     </row>
@@ -1645,7 +1741,10 @@
         <f>_xlfn.XLOOKUP(C34,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Accessories</v>
       </c>
-      <c r="H34" s="9"/>
+      <c r="H34" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C34,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I34" s="5"/>
       <c r="J34" s="1"/>
     </row>
@@ -1673,7 +1772,10 @@
         <f>_xlfn.XLOOKUP(C35,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H35" s="9"/>
+      <c r="H35" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C35,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I35" s="5"/>
       <c r="J35" s="1"/>
     </row>
@@ -1701,7 +1803,10 @@
         <f>_xlfn.XLOOKUP(C36,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H36" s="9"/>
+      <c r="H36" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C36,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I36" s="5"/>
       <c r="J36" s="1"/>
     </row>
@@ -1729,7 +1834,10 @@
         <f>_xlfn.XLOOKUP(C37,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H37" s="9"/>
+      <c r="H37" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C37,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I37" s="5"/>
       <c r="J37" s="1"/>
     </row>
@@ -1757,7 +1865,10 @@
         <f>_xlfn.XLOOKUP(C38,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Accessories</v>
       </c>
-      <c r="H38" s="9"/>
+      <c r="H38" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C38,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>StorePro</v>
+      </c>
       <c r="I38" s="5"/>
       <c r="J38" s="1"/>
     </row>
@@ -1785,7 +1896,10 @@
         <f>_xlfn.XLOOKUP(C39,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H39" s="9"/>
+      <c r="H39" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C39,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I39" s="5"/>
       <c r="J39" s="1"/>
     </row>
@@ -1813,7 +1927,10 @@
         <f>_xlfn.XLOOKUP(C40,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Furniture</v>
       </c>
-      <c r="H40" s="9"/>
+      <c r="H40" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C40,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>ComfortZone</v>
+      </c>
       <c r="I40" s="5"/>
       <c r="J40" s="1"/>
     </row>
@@ -1841,7 +1958,10 @@
         <f>_xlfn.XLOOKUP(C41,Sheet2!$A$2:$A$11,Sheet2!$C$2:$C$11)</f>
         <v>Electronics</v>
       </c>
-      <c r="H41" s="9"/>
+      <c r="H41" s="9" t="str">
+        <f>_xlfn.XLOOKUP(C41,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
+        <v>TechBrand</v>
+      </c>
       <c r="I41" s="5"/>
       <c r="J41" s="1"/>
     </row>

</xml_diff>

<commit_message>
Product Price is fetched according to Product ID from Sheet2  using xlookup formula
</commit_message>
<xml_diff>
--- a/Day 3/Day3_Practice_Data.xlsx
+++ b/Day 3/Day3_Practice_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{019F2CB7-FC5B-45D7-B083-5541DA50C83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00DE6499-174A-4901-86A7-D9B21DFC8A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{2C26B9A5-BE97-4C69-AF28-CEF3FE580AAE}"/>
   </bookViews>
@@ -753,7 +753,10 @@
         <f>_xlfn.XLOOKUP(C2,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I2" s="5"/>
+      <c r="I2" s="5">
+        <f>E2*_xlfn.XLOOKUP(C2,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>220000</v>
+      </c>
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -784,7 +787,10 @@
         <f>_xlfn.XLOOKUP(C3,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I3" s="5"/>
+      <c r="I3" s="5">
+        <f>E3*_xlfn.XLOOKUP(C3,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>1200</v>
+      </c>
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -815,7 +821,10 @@
         <f>_xlfn.XLOOKUP(C4,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I4" s="5"/>
+      <c r="I4" s="5">
+        <f>E4*_xlfn.XLOOKUP(C4,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>135000</v>
+      </c>
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -846,7 +855,10 @@
         <f>_xlfn.XLOOKUP(C5,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>WriteRight</v>
       </c>
-      <c r="I5" s="5"/>
+      <c r="I5" s="5">
+        <f>E5*_xlfn.XLOOKUP(C5,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>3600</v>
+      </c>
       <c r="J5" s="1"/>
     </row>
     <row r="6" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -877,7 +889,10 @@
         <f>_xlfn.XLOOKUP(C6,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I6" s="5"/>
+      <c r="I6" s="5">
+        <f>E6*_xlfn.XLOOKUP(C6,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>28000</v>
+      </c>
       <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -908,7 +923,10 @@
         <f>_xlfn.XLOOKUP(C7,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I7" s="5"/>
+      <c r="I7" s="5">
+        <f>E7*_xlfn.XLOOKUP(C7,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>140000</v>
+      </c>
       <c r="J7" s="1"/>
     </row>
     <row r="8" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -939,7 +957,10 @@
         <f>_xlfn.XLOOKUP(C8,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I8" s="5"/>
+      <c r="I8" s="5">
+        <f>E8*_xlfn.XLOOKUP(C8,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>140000</v>
+      </c>
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -970,7 +991,10 @@
         <f>_xlfn.XLOOKUP(C9,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I9" s="5"/>
+      <c r="I9" s="5">
+        <f>E9*_xlfn.XLOOKUP(C9,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>18000</v>
+      </c>
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1001,7 +1025,10 @@
         <f>_xlfn.XLOOKUP(C10,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I10" s="5"/>
+      <c r="I10" s="5">
+        <f>E10*_xlfn.XLOOKUP(C10,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>96000</v>
+      </c>
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1032,7 +1059,10 @@
         <f>_xlfn.XLOOKUP(C11,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I11" s="5"/>
+      <c r="I11" s="5">
+        <f>E11*_xlfn.XLOOKUP(C11,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>41800</v>
+      </c>
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1063,7 +1093,10 @@
         <f>_xlfn.XLOOKUP(C12,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I12" s="5"/>
+      <c r="I12" s="5">
+        <f>E12*_xlfn.XLOOKUP(C12,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>770000</v>
+      </c>
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1094,7 +1127,10 @@
         <f>_xlfn.XLOOKUP(C13,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I13" s="5"/>
+      <c r="I13" s="5">
+        <f>E13*_xlfn.XLOOKUP(C13,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>2400</v>
+      </c>
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1125,7 +1161,10 @@
         <f>_xlfn.XLOOKUP(C14,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I14" s="5"/>
+      <c r="I14" s="5">
+        <f>E14*_xlfn.XLOOKUP(C14,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>15000</v>
+      </c>
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1156,7 +1195,10 @@
         <f>_xlfn.XLOOKUP(C15,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>WriteRight</v>
       </c>
-      <c r="I15" s="5"/>
+      <c r="I15" s="5">
+        <f>E15*_xlfn.XLOOKUP(C15,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>1350</v>
+      </c>
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1187,7 +1229,10 @@
         <f>_xlfn.XLOOKUP(C16,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I16" s="5"/>
+      <c r="I16" s="5">
+        <f>E16*_xlfn.XLOOKUP(C16,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>24500</v>
+      </c>
       <c r="J16" s="1"/>
     </row>
     <row r="17" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1218,7 +1263,10 @@
         <f>_xlfn.XLOOKUP(C17,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I17" s="5"/>
+      <c r="I17" s="5">
+        <f>E17*_xlfn.XLOOKUP(C17,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>76500</v>
+      </c>
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1249,7 +1297,10 @@
         <f>_xlfn.XLOOKUP(C18,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>StorePro</v>
       </c>
-      <c r="I18" s="5"/>
+      <c r="I18" s="5">
+        <f>E18*_xlfn.XLOOKUP(C18,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>17000</v>
+      </c>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1280,7 +1331,10 @@
         <f>_xlfn.XLOOKUP(C19,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I19" s="5"/>
+      <c r="I19" s="5">
+        <f>E19*_xlfn.XLOOKUP(C19,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>32000</v>
+      </c>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1311,7 +1365,10 @@
         <f>_xlfn.XLOOKUP(C20,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I20" s="5"/>
+      <c r="I20" s="5">
+        <f>E20*_xlfn.XLOOKUP(C20,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>39600</v>
+      </c>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1342,7 +1399,10 @@
         <f>_xlfn.XLOOKUP(C21,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I21" s="5"/>
+      <c r="I21" s="5">
+        <f>E21*_xlfn.XLOOKUP(C21,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>385000</v>
+      </c>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1373,7 +1433,10 @@
         <f>_xlfn.XLOOKUP(C22,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I22" s="5"/>
+      <c r="I22" s="5">
+        <f>E22*_xlfn.XLOOKUP(C22,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>385000</v>
+      </c>
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1404,7 +1467,10 @@
         <f>_xlfn.XLOOKUP(C23,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I23" s="5"/>
+      <c r="I23" s="5">
+        <f>E23*_xlfn.XLOOKUP(C23,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>21600</v>
+      </c>
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1435,7 +1501,10 @@
         <f>_xlfn.XLOOKUP(C24,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I24" s="5"/>
+      <c r="I24" s="5">
+        <f>E24*_xlfn.XLOOKUP(C24,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>210000</v>
+      </c>
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1466,7 +1535,10 @@
         <f>_xlfn.XLOOKUP(C25,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I25" s="5"/>
+      <c r="I25" s="5">
+        <f>E25*_xlfn.XLOOKUP(C25,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>52500</v>
+      </c>
       <c r="J25" s="1"/>
     </row>
     <row r="26" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1497,7 +1569,10 @@
         <f>_xlfn.XLOOKUP(C26,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I26" s="5"/>
+      <c r="I26" s="5">
+        <f>E26*_xlfn.XLOOKUP(C26,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>532000</v>
+      </c>
       <c r="J26" s="1"/>
     </row>
     <row r="27" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1528,7 +1603,10 @@
         <f>_xlfn.XLOOKUP(C27,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I27" s="5"/>
+      <c r="I27" s="5">
+        <f>E27*_xlfn.XLOOKUP(C27,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>40500</v>
+      </c>
       <c r="J27" s="1"/>
     </row>
     <row r="28" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1559,7 +1637,10 @@
         <f>_xlfn.XLOOKUP(C28,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>StorePro</v>
       </c>
-      <c r="I28" s="5"/>
+      <c r="I28" s="5">
+        <f>E28*_xlfn.XLOOKUP(C28,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>850</v>
+      </c>
       <c r="J28" s="1"/>
     </row>
     <row r="29" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1590,7 +1671,10 @@
         <f>_xlfn.XLOOKUP(C29,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I29" s="5"/>
+      <c r="I29" s="5">
+        <f>E29*_xlfn.XLOOKUP(C29,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>192000</v>
+      </c>
       <c r="J29" s="1"/>
     </row>
     <row r="30" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1621,7 +1705,10 @@
         <f>_xlfn.XLOOKUP(C30,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I30" s="5"/>
+      <c r="I30" s="5">
+        <f>E30*_xlfn.XLOOKUP(C30,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>30800</v>
+      </c>
       <c r="J30" s="1"/>
     </row>
     <row r="31" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1652,7 +1739,10 @@
         <f>_xlfn.XLOOKUP(C31,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I31" s="5"/>
+      <c r="I31" s="5">
+        <f>E31*_xlfn.XLOOKUP(C31,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>605000</v>
+      </c>
       <c r="J31" s="1"/>
     </row>
     <row r="32" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1683,7 +1773,10 @@
         <f>_xlfn.XLOOKUP(C32,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I32" s="5"/>
+      <c r="I32" s="5">
+        <f>E32*_xlfn.XLOOKUP(C32,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>10800</v>
+      </c>
       <c r="J32" s="1"/>
     </row>
     <row r="33" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1714,7 +1807,10 @@
         <f>_xlfn.XLOOKUP(C33,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I33" s="5"/>
+      <c r="I33" s="5">
+        <f>E33*_xlfn.XLOOKUP(C33,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>75000</v>
+      </c>
       <c r="J33" s="1"/>
     </row>
     <row r="34" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1745,7 +1841,10 @@
         <f>_xlfn.XLOOKUP(C34,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I34" s="5"/>
+      <c r="I34" s="5">
+        <f>E34*_xlfn.XLOOKUP(C34,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>38500</v>
+      </c>
       <c r="J34" s="1"/>
     </row>
     <row r="35" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1776,7 +1875,10 @@
         <f>_xlfn.XLOOKUP(C35,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I35" s="5"/>
+      <c r="I35" s="5">
+        <f>E35*_xlfn.XLOOKUP(C35,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>112000</v>
+      </c>
       <c r="J35" s="1"/>
     </row>
     <row r="36" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1807,7 +1909,10 @@
         <f>_xlfn.XLOOKUP(C36,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I36" s="5"/>
+      <c r="I36" s="5">
+        <f>E36*_xlfn.XLOOKUP(C36,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>112000</v>
+      </c>
       <c r="J36" s="1"/>
     </row>
     <row r="37" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1838,7 +1943,10 @@
         <f>_xlfn.XLOOKUP(C37,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I37" s="5"/>
+      <c r="I37" s="5">
+        <f>E37*_xlfn.XLOOKUP(C37,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>13500</v>
+      </c>
       <c r="J37" s="1"/>
     </row>
     <row r="38" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1869,7 +1977,10 @@
         <f>_xlfn.XLOOKUP(C38,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>StorePro</v>
       </c>
-      <c r="I38" s="5"/>
+      <c r="I38" s="5">
+        <f>E38*_xlfn.XLOOKUP(C38,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>11050</v>
+      </c>
       <c r="J38" s="1"/>
     </row>
     <row r="39" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1900,7 +2011,10 @@
         <f>_xlfn.XLOOKUP(C39,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I39" s="5"/>
+      <c r="I39" s="5">
+        <f>E39*_xlfn.XLOOKUP(C39,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>128000</v>
+      </c>
       <c r="J39" s="1"/>
     </row>
     <row r="40" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1931,7 +2045,10 @@
         <f>_xlfn.XLOOKUP(C40,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>ComfortZone</v>
       </c>
-      <c r="I40" s="5"/>
+      <c r="I40" s="5">
+        <f>E40*_xlfn.XLOOKUP(C40,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>26400</v>
+      </c>
       <c r="J40" s="1"/>
     </row>
     <row r="41" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1962,7 +2079,10 @@
         <f>_xlfn.XLOOKUP(C41,Sheet2!$A$2:$A$11,Sheet2!$D$2:$D$11)</f>
         <v>TechBrand</v>
       </c>
-      <c r="I41" s="5"/>
+      <c r="I41" s="5">
+        <f>E41*_xlfn.XLOOKUP(C41,Sheet2!$A$2:$A$11,Sheet2!$E$2:$E$11)</f>
+        <v>660000</v>
+      </c>
       <c r="J41" s="1"/>
     </row>
   </sheetData>

</xml_diff>